<commit_message>
feat: 闭包支持 - Phase 1-5 完成
新增功能：
- functional/ 模块（closure.py, analyzer.py）
- LambdaExprNode AST 节点
- Lambda 表达式解析
- 闭包相关 IR 操作码

核心文件变更：
- src/zhc/functional/ - 新模块目录
- src/zhc/parser/ast_nodes.py - LambdaExprNode
- src/zhc/parser/parser.py - Lambda 解析
- src/zhc/ir/opcodes.py - 闭包操作码
- src/zhc/ir/ir_generator.py - Lambda IR 生成
</commit_message>
<xml_diff>
--- a/ZhC开发路线图 1.xlsx
+++ b/ZhC开发路线图 1.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="259">
   <si>
     <t>序号</t>
   </si>
@@ -751,7 +751,14 @@
     <t>异常捕获和处理</t>
   </si>
   <si>
-    <t>先提交 git，然后进行下一步开发。请把以下阶段的规划做成任务清单，逐个执行。 要求：每个任务开始前，必须先对照项目代码进行二次分析，核查开发文档的正确性，并挑选出有效的开发需求，进行开发。</t>
+    <t>待完成
+LLVM EH intrinsics 集成（landingpad, resume）
+IR Generator 中生成异常处理 IR 节点
+与现有变量声明/作用域的完整集成
+单元测试</t>
+  </si>
+  <si>
+    <t>先提交 git，然后进行下一步开发。请把以下阶段的规划做成任务清单，逐个执行。 要求：每个任务开始前，必须先对照Zhc项目代码进行二次分析，核查开发文档的正确性，并挑选出有效的开发需求，进行开发。</t>
   </si>
   <si>
     <t>异常类型系统</t>
@@ -770,6 +777,59 @@
   </si>
   <si>
     <t>请把以下阶段的规划做成任务清单，逐个执行。</t>
+  </si>
+  <si>
+    <r>
+      <t>阶段</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">6: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>高级特性</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>自定义异常</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>并集成到语义分析器</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/IR</t>
+    </r>
+  </si>
+  <si>
+    <t>自定义异常类型支持，集成</t>
   </si>
   <si>
     <t>函数式</t>
@@ -1616,7 +1676,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1630,6 +1690,11 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2163,7 +2228,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N85"/>
+  <dimension ref="A1:O86"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2173,10 +2238,12 @@
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="9" width="10" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="39.84375" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" spans="1:14">
+    <row r="1" ht="18" customHeight="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2204,8 +2271,9 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2234,7 +2302,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:15">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2262,15 +2330,15 @@
       <c r="I3" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
-    </row>
-    <row r="4" spans="1:14">
+      <c r="O3" s="4"/>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2298,13 +2366,13 @@
       <c r="I4" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
-    </row>
-    <row r="5" spans="1:14">
+      <c r="O4" s="4"/>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2332,13 +2400,13 @@
       <c r="I5" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
-    </row>
-    <row r="6" spans="1:14">
+      <c r="O5" s="4"/>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2366,13 +2434,13 @@
       <c r="I6" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
-    </row>
-    <row r="7" spans="1:14">
+      <c r="O6" s="4"/>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2400,13 +2468,13 @@
       <c r="I7" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
-    </row>
-    <row r="8" spans="1:14">
+      <c r="O7" s="4"/>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2434,13 +2502,13 @@
       <c r="I8" t="s">
         <v>15</v>
       </c>
-      <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
-    </row>
-    <row r="9" spans="1:14">
+      <c r="O8" s="4"/>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2468,13 +2536,13 @@
       <c r="I9" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
-    </row>
-    <row r="10" spans="1:14">
+      <c r="O9" s="4"/>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2503,7 +2571,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:15">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2532,7 +2600,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:15">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2561,7 +2629,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:15">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2590,7 +2658,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:15">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2619,7 +2687,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:15">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2648,7 +2716,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:15">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3605,7 +3673,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:11">
+    <row r="49" spans="1:12">
       <c r="A49">
         <v>48</v>
       </c>
@@ -3634,7 +3702,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:11">
+    <row r="50" spans="1:12">
       <c r="A50">
         <v>49</v>
       </c>
@@ -3663,7 +3731,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:11">
+    <row r="51" spans="1:12">
       <c r="A51">
         <v>50</v>
       </c>
@@ -3692,7 +3760,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:11">
+    <row r="52" spans="1:12">
       <c r="A52">
         <v>51</v>
       </c>
@@ -3721,7 +3789,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="1:11">
+    <row r="53" spans="1:12">
       <c r="A53">
         <v>52</v>
       </c>
@@ -3750,7 +3818,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:11">
+    <row r="54" spans="1:12">
       <c r="A54">
         <v>53</v>
       </c>
@@ -3779,7 +3847,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:11">
+    <row r="55" spans="1:12">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3808,7 +3876,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:11">
+    <row r="56" spans="1:12">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3837,7 +3905,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="1:11">
+    <row r="57" spans="1:12">
       <c r="A57">
         <v>56</v>
       </c>
@@ -3866,7 +3934,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="58" spans="1:11">
+    <row r="58" spans="1:12">
       <c r="A58">
         <v>57</v>
       </c>
@@ -3895,7 +3963,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:11">
+    <row r="59" spans="1:12">
       <c r="A59">
         <v>58</v>
       </c>
@@ -3924,7 +3992,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="60" spans="1:11">
+    <row r="60" spans="1:12">
       <c r="A60">
         <v>59</v>
       </c>
@@ -3953,7 +4021,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:11">
+    <row r="61" ht="15" customHeight="1" spans="1:12">
       <c r="A61">
         <v>60</v>
       </c>
@@ -3978,14 +4046,14 @@
       <c r="H61" t="s">
         <v>14</v>
       </c>
-      <c r="I61" t="s">
-        <v>15</v>
-      </c>
-      <c r="J61" t="s">
+      <c r="I61" s="9" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="62" spans="1:11">
+      <c r="K61" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="62" ht="21" customHeight="1" spans="1:12">
       <c r="A62">
         <v>61</v>
       </c>
@@ -3999,25 +4067,23 @@
         <v>183</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G62">
         <v>3</v>
       </c>
       <c r="H62" t="s">
-        <v>189</v>
-      </c>
-      <c r="I62" t="s">
-        <v>15</v>
-      </c>
-      <c r="J62" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11">
+        <v>190</v>
+      </c>
+      <c r="I62" s="9"/>
+      <c r="K62" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="63" ht="17" customHeight="1" spans="1:12">
       <c r="A63">
         <v>62</v>
       </c>
@@ -4031,65 +4097,49 @@
         <v>183</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G63">
         <v>3</v>
       </c>
       <c r="H63" t="s">
-        <v>189</v>
-      </c>
-      <c r="I63" t="s">
-        <v>15</v>
-      </c>
-      <c r="J63" t="s">
-        <v>186</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="I63" s="9"/>
       <c r="K63" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11">
-      <c r="A64">
-        <v>63</v>
-      </c>
-      <c r="B64" t="s">
-        <v>181</v>
+        <v>187</v>
+      </c>
+      <c r="L63" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="64" ht="17" spans="1:12">
+      <c r="B64" s="10" t="s">
+        <v>194</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>182</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="E64" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="F64" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="E64" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="G64">
-        <v>7</v>
-      </c>
-      <c r="H64" t="s">
-        <v>14</v>
-      </c>
-      <c r="I64" t="s">
-        <v>15</v>
-      </c>
-      <c r="J64" t="s">
-        <v>186</v>
-      </c>
+      <c r="F64" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="I64" s="9"/>
       <c r="K64" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12">
       <c r="A65">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" t="s">
         <v>181</v>
@@ -4098,16 +4148,16 @@
         <v>182</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F65" s="8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G65">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H65" t="s">
         <v>14</v>
@@ -4115,16 +4165,16 @@
       <c r="I65" t="s">
         <v>15</v>
       </c>
-      <c r="J65" t="s">
-        <v>186</v>
-      </c>
       <c r="K65" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11">
+        <v>187</v>
+      </c>
+      <c r="L65" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12">
       <c r="A66">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B66" t="s">
         <v>181</v>
@@ -4133,16 +4183,16 @@
         <v>182</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>46</v>
+        <v>197</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G66">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H66" t="s">
         <v>14</v>
@@ -4150,13 +4200,16 @@
       <c r="I66" t="s">
         <v>15</v>
       </c>
-      <c r="J66" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11">
+      <c r="K66" t="s">
+        <v>187</v>
+      </c>
+      <c r="L66" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12">
       <c r="A67">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B67" t="s">
         <v>181</v>
@@ -4168,10 +4221,10 @@
         <v>46</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G67">
         <v>4</v>
@@ -4182,13 +4235,13 @@
       <c r="I67" t="s">
         <v>15</v>
       </c>
-      <c r="J67" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11">
+      <c r="K67" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12">
       <c r="A68">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B68" t="s">
         <v>181</v>
@@ -4197,16 +4250,16 @@
         <v>182</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>204</v>
+        <v>46</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G68">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H68" t="s">
         <v>14</v>
@@ -4214,13 +4267,13 @@
       <c r="I68" t="s">
         <v>15</v>
       </c>
-      <c r="J68" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11">
+      <c r="K68" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12">
       <c r="A69">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B69" t="s">
         <v>181</v>
@@ -4229,30 +4282,30 @@
         <v>182</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F69" s="8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G69">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H69" t="s">
-        <v>209</v>
+        <v>14</v>
       </c>
       <c r="I69" t="s">
         <v>15</v>
       </c>
-      <c r="J69" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11">
+      <c r="K69" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12">
       <c r="A70">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B70" t="s">
         <v>181</v>
@@ -4261,30 +4314,30 @@
         <v>182</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>180</v>
+        <v>211</v>
       </c>
       <c r="F70" s="8" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H70" t="s">
-        <v>14</v>
+        <v>213</v>
       </c>
       <c r="I70" t="s">
         <v>15</v>
       </c>
-      <c r="J70" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11">
+      <c r="K70" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12">
       <c r="A71">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B71" t="s">
         <v>181</v>
@@ -4293,16 +4346,16 @@
         <v>182</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>212</v>
+        <v>180</v>
       </c>
       <c r="F71" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G71">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H71" t="s">
         <v>14</v>
@@ -4310,13 +4363,13 @@
       <c r="I71" t="s">
         <v>15</v>
       </c>
-      <c r="J71" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11">
+      <c r="K71" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12">
       <c r="A72">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B72" t="s">
         <v>181</v>
@@ -4325,30 +4378,30 @@
         <v>182</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F72" s="8" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G72">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H72" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
       <c r="I72" t="s">
         <v>15</v>
       </c>
-      <c r="J72" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11">
+      <c r="K72" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12">
       <c r="A73">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B73" t="s">
         <v>181</v>
@@ -4357,161 +4410,164 @@
         <v>182</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G73">
+        <v>4</v>
+      </c>
+      <c r="H73" t="s">
+        <v>220</v>
+      </c>
+      <c r="I73" t="s">
+        <v>15</v>
+      </c>
+      <c r="K73" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12">
+      <c r="A74">
+        <v>72</v>
+      </c>
+      <c r="B74" t="s">
+        <v>181</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="F74" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="G74">
         <v>3</v>
       </c>
-      <c r="H73" t="s">
-        <v>216</v>
-      </c>
-      <c r="I73" t="s">
-        <v>15</v>
-      </c>
-      <c r="J73" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11">
-      <c r="A74">
+      <c r="H74" t="s">
+        <v>220</v>
+      </c>
+      <c r="I74" t="s">
+        <v>15</v>
+      </c>
+      <c r="K74" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12">
+      <c r="A75">
         <v>73</v>
       </c>
-      <c r="B74" t="s">
-        <v>219</v>
-      </c>
-      <c r="C74" t="s">
-        <v>220</v>
-      </c>
-      <c r="D74" t="s">
-        <v>221</v>
-      </c>
-      <c r="E74" t="s">
-        <v>222</v>
-      </c>
-      <c r="F74" t="s">
+      <c r="B75" t="s">
         <v>223</v>
       </c>
-      <c r="G74">
+      <c r="C75" t="s">
+        <v>224</v>
+      </c>
+      <c r="D75" t="s">
+        <v>225</v>
+      </c>
+      <c r="E75" t="s">
+        <v>226</v>
+      </c>
+      <c r="F75" t="s">
+        <v>227</v>
+      </c>
+      <c r="G75">
         <v>5</v>
       </c>
-      <c r="H74" t="s">
+      <c r="H75" t="s">
         <v>14</v>
       </c>
-      <c r="I74" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11">
-      <c r="A75">
+      <c r="I75" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12">
+      <c r="A76">
         <v>74</v>
       </c>
-      <c r="B75" t="s">
-        <v>219</v>
-      </c>
-      <c r="C75" t="s">
-        <v>220</v>
-      </c>
-      <c r="D75" t="s">
-        <v>221</v>
-      </c>
-      <c r="E75" t="s">
+      <c r="B76" t="s">
+        <v>223</v>
+      </c>
+      <c r="C76" t="s">
         <v>224</v>
       </c>
-      <c r="F75" t="s">
+      <c r="D76" t="s">
         <v>225</v>
       </c>
-      <c r="G75">
+      <c r="E76" t="s">
+        <v>228</v>
+      </c>
+      <c r="F76" t="s">
+        <v>229</v>
+      </c>
+      <c r="G76">
         <v>4</v>
       </c>
-      <c r="H75" t="s">
-        <v>226</v>
-      </c>
-      <c r="I75" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11">
-      <c r="A76">
+      <c r="H76" t="s">
+        <v>230</v>
+      </c>
+      <c r="I76" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12">
+      <c r="A77">
         <v>75</v>
       </c>
-      <c r="B76" t="s">
-        <v>219</v>
-      </c>
-      <c r="C76" t="s">
-        <v>220</v>
-      </c>
-      <c r="D76" t="s">
-        <v>221</v>
-      </c>
-      <c r="E76" t="s">
-        <v>227</v>
-      </c>
-      <c r="F76" t="s">
-        <v>228</v>
-      </c>
-      <c r="G76">
+      <c r="B77" t="s">
+        <v>223</v>
+      </c>
+      <c r="C77" t="s">
+        <v>224</v>
+      </c>
+      <c r="D77" t="s">
+        <v>225</v>
+      </c>
+      <c r="E77" t="s">
+        <v>231</v>
+      </c>
+      <c r="F77" t="s">
+        <v>232</v>
+      </c>
+      <c r="G77">
         <v>5</v>
       </c>
-      <c r="H76" t="s">
-        <v>226</v>
-      </c>
-      <c r="I76" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11">
-      <c r="A77">
+      <c r="H77" t="s">
+        <v>230</v>
+      </c>
+      <c r="I77" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12">
+      <c r="A78">
         <v>76</v>
       </c>
-      <c r="B77" t="s">
-        <v>219</v>
-      </c>
-      <c r="C77" t="s">
-        <v>220</v>
-      </c>
-      <c r="D77" t="s">
-        <v>229</v>
-      </c>
-      <c r="E77" t="s">
-        <v>230</v>
-      </c>
-      <c r="F77" t="s">
-        <v>231</v>
-      </c>
-      <c r="G77">
-        <v>7</v>
-      </c>
-      <c r="H77" t="s">
-        <v>14</v>
-      </c>
-      <c r="I77" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11">
-      <c r="A78">
-        <v>77</v>
-      </c>
       <c r="B78" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C78" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="D78" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E78" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F78" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G78">
         <v>7</v>
@@ -4523,27 +4579,27 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:11">
+    <row r="79" spans="1:12">
       <c r="A79">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B79" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C79" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="D79" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E79" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F79" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G79">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H79" t="s">
         <v>14</v>
@@ -4552,27 +4608,27 @@
         <v>15</v>
       </c>
     </row>
-    <row r="80" spans="1:11">
+    <row r="80" spans="1:12">
       <c r="A80">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B80" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="C80" t="s">
+        <v>224</v>
+      </c>
+      <c r="D80" t="s">
         <v>239</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>240</v>
       </c>
-      <c r="E80" t="s">
+      <c r="F80" t="s">
         <v>241</v>
       </c>
-      <c r="F80" t="s">
-        <v>242</v>
-      </c>
       <c r="G80">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H80" t="s">
         <v>14</v>
@@ -4583,25 +4639,25 @@
     </row>
     <row r="81" spans="1:9">
       <c r="A81">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B81" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C81" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D81" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="E81" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F81" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G81">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H81" t="s">
         <v>14</v>
@@ -4612,25 +4668,25 @@
     </row>
     <row r="82" spans="1:9">
       <c r="A82">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C82" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D82" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="E82" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F82" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G82">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H82" t="s">
         <v>14</v>
@@ -4641,25 +4697,25 @@
     </row>
     <row r="83" spans="1:9">
       <c r="A83">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B83" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C83" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D83" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E83" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F83" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G83">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H83" t="s">
         <v>14</v>
@@ -4670,28 +4726,28 @@
     </row>
     <row r="84" spans="1:9">
       <c r="A84">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B84" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C84" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D84" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="E84" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F84" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="G84">
         <v>3</v>
       </c>
       <c r="H84" t="s">
-        <v>252</v>
+        <v>14</v>
       </c>
       <c r="I84" t="s">
         <v>15</v>
@@ -4699,36 +4755,65 @@
     </row>
     <row r="85" spans="1:9">
       <c r="A85">
+        <v>83</v>
+      </c>
+      <c r="B85" t="s">
+        <v>242</v>
+      </c>
+      <c r="C85" t="s">
+        <v>243</v>
+      </c>
+      <c r="D85" t="s">
+        <v>251</v>
+      </c>
+      <c r="E85" t="s">
+        <v>254</v>
+      </c>
+      <c r="F85" t="s">
+        <v>255</v>
+      </c>
+      <c r="G85">
+        <v>3</v>
+      </c>
+      <c r="H85" t="s">
+        <v>256</v>
+      </c>
+      <c r="I85" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9">
+      <c r="A86">
         <v>84</v>
       </c>
-      <c r="B85" t="s">
-        <v>238</v>
-      </c>
-      <c r="C85" t="s">
-        <v>239</v>
-      </c>
-      <c r="D85" t="s">
-        <v>247</v>
-      </c>
-      <c r="E85" t="s">
-        <v>253</v>
-      </c>
-      <c r="F85" t="s">
-        <v>254</v>
-      </c>
-      <c r="G85">
+      <c r="B86" t="s">
+        <v>242</v>
+      </c>
+      <c r="C86" t="s">
+        <v>243</v>
+      </c>
+      <c r="D86" t="s">
+        <v>251</v>
+      </c>
+      <c r="E86" t="s">
+        <v>257</v>
+      </c>
+      <c r="F86" t="s">
+        <v>258</v>
+      </c>
+      <c r="G86">
         <v>5</v>
       </c>
-      <c r="H85" t="s">
-        <v>252</v>
-      </c>
-      <c r="I85" t="s">
+      <c r="H86" t="s">
+        <v>256</v>
+      </c>
+      <c r="I86" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="J3:N9"/>
+    <mergeCell ref="K3:O9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
feat: 模式匹配 IR/Backend 集成 + ASTVisitor 同步修复
- 添加模式匹配 IR 操作码 (MATCH_EXPR, MATCH_CASE, PATTERN_BIND 等)
- IRGenerator 添加 visit_match_expr/visit_match_case 抽象方法实现
- 新增 pattern_strategies.py 后端策略模块
- ASTNodes 添加 MatchExprNode/MatchCaseNode 节点
- 同步修复所有 ASTVisitor 继承类的抽象方法
- 清理未使用的导入和变量 (Lint 修复)

测试: 3511 passed / 4 skipped / 3 xpassed
</commit_message>
<xml_diff>
--- a/ZhC开发路线图 1.xlsx
+++ b/ZhC开发路线图 1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29400" windowHeight="12320"/>
+    <workbookView windowWidth="17720" windowHeight="7440"/>
   </bookViews>
   <sheets>
     <sheet name="开发路线图" sheetId="1" r:id="rId1"/>
@@ -87,6 +87,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>请把以下阶段的规划做成任务清单，逐个执行。</t>
     </r>
     <r>
@@ -773,6 +778,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>阶段</t>
     </r>
     <r>
@@ -794,6 +804,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>自定义异常</t>
     </r>
     <r>
@@ -888,40 +903,40 @@
     <t>运行时类型信息</t>
   </si>
   <si>
+    <t>我们需要程序编译器专家的帮助，帮助我们进行下一步开发。把以下阶段的规划做成任务清单，逐个执行。 要求：每个任务开始前，必须先对照Zhc项目代码进行二次分析，核查开发需求的正确性，并挑选出有效的开发需求，进行开发。</t>
+  </si>
+  <si>
+    <t>运行时类型检查</t>
+  </si>
+  <si>
+    <t>动态类型检查</t>
+  </si>
+  <si>
+    <t>序号70</t>
+  </si>
+  <si>
+    <t>动态类型转换</t>
+  </si>
+  <si>
+    <t>安全的类型转换</t>
+  </si>
+  <si>
+    <t>阶段7: 后端支持</t>
+  </si>
+  <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>WASM</t>
+  </si>
+  <si>
+    <t>WASM 特定优化</t>
+  </si>
+  <si>
+    <t>WebAssembly 优化</t>
+  </si>
+  <si>
     <t>待开发</t>
-  </si>
-  <si>
-    <t>我们需要程序编译器专家的帮助，帮助我们进行下一步开发。把以下阶段的规划做成任务清单，逐个执行。 要求：每个任务开始前，必须先对照Zhc项目代码进行二次分析，核查开发需求的正确性，并挑选出有效的开发需求，进行开发。</t>
-  </si>
-  <si>
-    <t>运行时类型检查</t>
-  </si>
-  <si>
-    <t>动态类型检查</t>
-  </si>
-  <si>
-    <t>序号70</t>
-  </si>
-  <si>
-    <t>动态类型转换</t>
-  </si>
-  <si>
-    <t>安全的类型转换</t>
-  </si>
-  <si>
-    <t>阶段7: 后端支持</t>
-  </si>
-  <si>
-    <t>P6</t>
-  </si>
-  <si>
-    <t>WASM</t>
-  </si>
-  <si>
-    <t>WASM 特定优化</t>
-  </si>
-  <si>
-    <t>WebAssembly 优化</t>
   </si>
   <si>
     <t>WASI 系统调用</t>
@@ -4401,11 +4416,11 @@
       <c r="H72" t="s">
         <v>14</v>
       </c>
-      <c r="I72" s="11" t="s">
+      <c r="I72" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K72" t="s">
         <v>217</v>
-      </c>
-      <c r="K72" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -4422,22 +4437,22 @@
         <v>214</v>
       </c>
       <c r="E73" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="F73" s="9" t="s">
         <v>219</v>
-      </c>
-      <c r="F73" s="9" t="s">
-        <v>220</v>
       </c>
       <c r="G73">
         <v>4</v>
       </c>
       <c r="H73" t="s">
-        <v>221</v>
-      </c>
-      <c r="I73" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K73" t="s">
         <v>217</v>
-      </c>
-      <c r="K73" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -4454,22 +4469,22 @@
         <v>214</v>
       </c>
       <c r="E74" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="F74" s="9" t="s">
         <v>222</v>
-      </c>
-      <c r="F74" s="9" t="s">
-        <v>223</v>
       </c>
       <c r="G74">
         <v>3</v>
       </c>
       <c r="H74" t="s">
-        <v>221</v>
-      </c>
-      <c r="I74" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K74" t="s">
         <v>217</v>
-      </c>
-      <c r="K74" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -4477,19 +4492,19 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
+        <v>223</v>
+      </c>
+      <c r="C75" t="s">
         <v>224</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>225</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>226</v>
       </c>
-      <c r="E75" t="s">
+      <c r="F75" t="s">
         <v>227</v>
-      </c>
-      <c r="F75" t="s">
-        <v>228</v>
       </c>
       <c r="G75">
         <v>5</v>
@@ -4498,10 +4513,10 @@
         <v>14</v>
       </c>
       <c r="I75" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K75" t="s">
         <v>217</v>
-      </c>
-      <c r="K75" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -4509,13 +4524,13 @@
         <v>74</v>
       </c>
       <c r="B76" t="s">
+        <v>223</v>
+      </c>
+      <c r="C76" t="s">
         <v>224</v>
       </c>
-      <c r="C76" t="s">
+      <c r="D76" t="s">
         <v>225</v>
-      </c>
-      <c r="D76" t="s">
-        <v>226</v>
       </c>
       <c r="E76" t="s">
         <v>229</v>
@@ -4530,10 +4545,10 @@
         <v>231</v>
       </c>
       <c r="I76" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K76" t="s">
         <v>217</v>
-      </c>
-      <c r="K76" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -4541,13 +4556,13 @@
         <v>75</v>
       </c>
       <c r="B77" t="s">
+        <v>223</v>
+      </c>
+      <c r="C77" t="s">
         <v>224</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>225</v>
-      </c>
-      <c r="D77" t="s">
-        <v>226</v>
       </c>
       <c r="E77" t="s">
         <v>232</v>
@@ -4562,10 +4577,10 @@
         <v>231</v>
       </c>
       <c r="I77" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K77" t="s">
         <v>217</v>
-      </c>
-      <c r="K77" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -4573,10 +4588,10 @@
         <v>76</v>
       </c>
       <c r="B78" t="s">
+        <v>223</v>
+      </c>
+      <c r="C78" t="s">
         <v>224</v>
-      </c>
-      <c r="C78" t="s">
-        <v>225</v>
       </c>
       <c r="D78" t="s">
         <v>234</v>
@@ -4594,10 +4609,10 @@
         <v>14</v>
       </c>
       <c r="I78" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K78" t="s">
         <v>217</v>
-      </c>
-      <c r="K78" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -4605,10 +4620,10 @@
         <v>77</v>
       </c>
       <c r="B79" t="s">
+        <v>223</v>
+      </c>
+      <c r="C79" t="s">
         <v>224</v>
-      </c>
-      <c r="C79" t="s">
-        <v>225</v>
       </c>
       <c r="D79" t="s">
         <v>237</v>
@@ -4626,10 +4641,10 @@
         <v>14</v>
       </c>
       <c r="I79" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K79" t="s">
         <v>217</v>
-      </c>
-      <c r="K79" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="80" spans="1:12">
@@ -4637,10 +4652,10 @@
         <v>78</v>
       </c>
       <c r="B80" t="s">
+        <v>223</v>
+      </c>
+      <c r="C80" t="s">
         <v>224</v>
-      </c>
-      <c r="C80" t="s">
-        <v>225</v>
       </c>
       <c r="D80" t="s">
         <v>240</v>
@@ -4658,10 +4673,10 @@
         <v>14</v>
       </c>
       <c r="I80" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K80" t="s">
         <v>217</v>
-      </c>
-      <c r="K80" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="81" spans="1:11">
@@ -4690,10 +4705,10 @@
         <v>14</v>
       </c>
       <c r="I81" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K81" t="s">
         <v>217</v>
-      </c>
-      <c r="K81" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="82" spans="1:11">
@@ -4722,10 +4737,10 @@
         <v>14</v>
       </c>
       <c r="I82" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K82" t="s">
         <v>217</v>
-      </c>
-      <c r="K82" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="83" spans="1:11">
@@ -4754,10 +4769,10 @@
         <v>14</v>
       </c>
       <c r="I83" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K83" t="s">
         <v>217</v>
-      </c>
-      <c r="K83" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="84" spans="1:11">
@@ -4786,10 +4801,10 @@
         <v>14</v>
       </c>
       <c r="I84" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K84" t="s">
         <v>217</v>
-      </c>
-      <c r="K84" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="85" spans="1:11">
@@ -4818,10 +4833,10 @@
         <v>257</v>
       </c>
       <c r="I85" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K85" t="s">
         <v>217</v>
-      </c>
-      <c r="K85" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="86" spans="1:11">
@@ -4850,10 +4865,10 @@
         <v>257</v>
       </c>
       <c r="I86" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="K86" t="s">
         <v>217</v>
-      </c>
-      <c r="K86" t="s">
-        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>